<commit_message>
feat(xlsx): complete fixture suite to R:5† — 21 fixtures, gen_fixtures binary, COVERAGE.md
Adds a fixture generator binary (gen_fixtures) for rescribe-read-xlsx that
programmatically builds XLSX files using ooxml-sml's WorkbookBuilder/SheetBuilder API.

New/updated fixtures (21 total):
  Basic: basic (regen), multi-sheet (regen), formula (regen)
  Cell types: numbers, booleans, cell-types-mixed
  Structural: merged-cells, freeze-pane, auto-filter, column-widths, row-heights
  Cell interactions: hyperlinks, comments
  Adversarial: adv-empty-workbook, adv-empty-sheet, adv-malformed-zip, adv-empty-bytes
  Pathological: path-many-rows, path-many-columns, path-many-sheets
  Composition: mixed-content

COVERAGE.md updated with [lib] markers for library-limited items (cell formatting,
date types, named ranges, hidden sheets — not represented in IR).

Promotes xlsx: R:4†→R:5† in format-audit.md.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/xlsx/basic/input.xlsx
+++ b/fixtures/xlsx/basic/input.xlsx
@@ -8,15 +8,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
-  <si>
-    <t>Alice</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Value</t>
   </si>
   <si>
-    <t>42</t>
+    <t>Alice</t>
   </si>
   <si>
     <t>Name</t>
@@ -29,18 +26,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
-      <c r="B2" t="s">
-        <v>2</v>
+      <c r="B2">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>